<commit_message>
Import Excel function for users and buildings
</commit_message>
<xml_diff>
--- a/sample_users.xlsx
+++ b/sample_users.xlsx
@@ -398,14 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F9"/>
-  <cols>
-    <col min="1" max="1" width="12.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="24.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -429,16 +421,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>James</v>
+        <v>Wei Jie</v>
       </c>
       <c r="B2" t="str">
-        <v>Tan</v>
+        <v>Ong</v>
       </c>
       <c r="C2" t="str">
-        <v>james.tan@cbre.com</v>
+        <v>weijie.ong.46053@cbre.com</v>
       </c>
       <c r="D2" t="str">
-        <v>+65 9123 4567</v>
+        <v>+65 8123 4567</v>
       </c>
       <c r="E2" t="str">
         <v>FSM</v>
@@ -449,16 +441,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Sarah</v>
+        <v>Hui Min</v>
       </c>
       <c r="B3" t="str">
-        <v>Lim</v>
+        <v>Teo</v>
       </c>
       <c r="C3" t="str">
-        <v>sarah.lim@cbre.com</v>
+        <v>huimin.teo.46053@cbre.com</v>
       </c>
       <c r="D3" t="str">
-        <v>+65 9234 5678</v>
+        <v>+65 8234 5678</v>
       </c>
       <c r="E3" t="str">
         <v>FSM</v>
@@ -469,16 +461,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>David</v>
+        <v>Kai Xuan</v>
       </c>
       <c r="B4" t="str">
-        <v>Ng</v>
+        <v>Lee</v>
       </c>
       <c r="C4" t="str">
-        <v>david.ng@cbre.com</v>
+        <v>kaixuan.lee.46053@cbre.com</v>
       </c>
       <c r="D4" t="str">
-        <v>+65 9345 6789</v>
+        <v>+65 8345 6789</v>
       </c>
       <c r="E4" t="str">
         <v>FSM</v>
@@ -489,16 +481,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Priya</v>
+        <v>Ravi</v>
       </c>
       <c r="B5" t="str">
-        <v>Rajan</v>
+        <v>Kumar</v>
       </c>
       <c r="C5" t="str">
-        <v>priya.rajan@cbre.com</v>
+        <v>ravi.kumar.46053@cbre.com</v>
       </c>
       <c r="D5" t="str">
-        <v>+65 9456 7890</v>
+        <v>+65 8456 7890</v>
       </c>
       <c r="E5" t="str">
         <v>FSM</v>
@@ -509,16 +501,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Michael</v>
+        <v>Nur</v>
       </c>
       <c r="B6" t="str">
-        <v>Chen</v>
+        <v>Aisyah</v>
       </c>
       <c r="C6" t="str">
-        <v>michael.chen@cbre.com</v>
+        <v>nur.aisyah.46053@cbre.com</v>
       </c>
       <c r="D6" t="str">
-        <v>+65 9567 8901</v>
+        <v>+65 8567 8901</v>
       </c>
       <c r="E6" t="str">
         <v>FSM</v>
@@ -529,16 +521,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Linda</v>
+        <v>Benjamin</v>
       </c>
       <c r="B7" t="str">
-        <v>Wong</v>
+        <v>Goh</v>
       </c>
       <c r="C7" t="str">
-        <v>linda.wong@client.com</v>
+        <v>benjamin.goh.46053@client.com</v>
       </c>
       <c r="D7" t="str">
-        <v>+65 9678 9012</v>
+        <v>+65 8678 9012</v>
       </c>
       <c r="E7" t="str">
         <v>Customer</v>
@@ -549,16 +541,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Robert</v>
+        <v>Farah</v>
       </c>
       <c r="B8" t="str">
-        <v>Koh</v>
+        <v>Ibrahim</v>
       </c>
       <c r="C8" t="str">
-        <v>robert.koh@client.com</v>
+        <v>farah.ibrahim.46053@client.com</v>
       </c>
       <c r="D8" t="str">
-        <v>+65 9789 0123</v>
+        <v>+65 8789 0123</v>
       </c>
       <c r="E8" t="str">
         <v>Customer</v>
@@ -569,16 +561,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Angela</v>
+        <v>Marcus</v>
       </c>
       <c r="B9" t="str">
-        <v>Seah</v>
+        <v>Tan</v>
       </c>
       <c r="C9" t="str">
-        <v>angela.seah@client.com</v>
+        <v>marcus.tan.46053@client.com</v>
       </c>
       <c r="D9" t="str">
-        <v>+65 9890 1234</v>
+        <v>+65 8890 1234</v>
       </c>
       <c r="E9" t="str">
         <v>Customer</v>

</xml_diff>